<commit_message>
f29h85x: All: Update MCAL package
- Update MCAL package

Fixes: MCAL-33825

Signed-off-by: Shyalu Sivan <s-sivan@ti.com>
</commit_message>
<xml_diff>
--- a/docs/Test_Report/TestPlanExecutionReport.xlsx
+++ b/docs/Test_Report/TestPlanExecutionReport.xlsx
@@ -734,7 +734,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2025-11-19 05:58:54.356285-06:00 CDT</t>
+          <t>2025-11-20 04:14:42.908612-06:00 CDT</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>MCAL-28162,MCAL-28163,MCAL-25808,MCAL-25806,MCAL-25807,MCAL-25801,MCAL-25799,MCAL-25797,MCAL-25811,MCAL-25810,MCAL-25809,MCAL-25804,MCAL-25803,MCAL-25802,MCAL-25798,MCAL-25796,MCAL-25805,MCAL-25800,MCAL-28161,MCAL-25820,MCAL-28165,MCAL-28164,MCAL-25812</t>
+          <t>MCAL-28162,MCAL-28163,MCAL-25808,MCAL-25806,MCAL-25807,MCAL-25801,MCAL-25799,MCAL-25800,MCAL-25820,MCAL-28165,MCAL-28164,MCAL-25797,MCAL-25812,MCAL-25811,MCAL-25810,MCAL-28161,MCAL-25809,MCAL-25804,MCAL-25803,MCAL-25802,MCAL-25798,MCAL-25796,MCAL-25805</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>MCAL-25814,MCAL-25721,MCAL-25720,MCAL-25717,MCAL-25712,MCAL-25711,MCAL-25701,MCAL-25715,MCAL-25704,MCAL-25702,MCAL-25716,MCAL-25718,MCAL-25706,MCAL-25709,MCAL-25708,MCAL-25707,MCAL-25813,MCAL-25710,MCAL-25705,MCAL-25714,MCAL-25713,MCAL-25723,MCAL-25731,MCAL-25727,MCAL-25726,MCAL-25724,MCAL-25725,MCAL-28133,MCAL-25703,MCAL-25824,MCAL-25823,MCAL-25732,MCAL-25722,MCAL-25719,MCAL-28135,MCAL-25825,MCAL-28134,MCAL-25822,MCAL-25730,MCAL-25729,MCAL-25728</t>
+          <t>MCAL-25814,MCAL-25721,MCAL-25720,MCAL-25717,MCAL-25712,MCAL-25711,MCAL-25701,MCAL-25715,MCAL-25704,MCAL-25702,MCAL-25716,MCAL-25718,MCAL-25706,MCAL-25709,MCAL-25708,MCAL-25707,MCAL-25813,MCAL-25723,MCAL-25731,MCAL-25727,MCAL-25726,MCAL-25724,MCAL-25725,MCAL-28133,MCAL-25703,MCAL-25824,MCAL-25823,MCAL-25732,MCAL-25722,MCAL-25719,MCAL-28135,MCAL-25825,MCAL-25710,MCAL-25705,MCAL-25714,MCAL-25713,MCAL-28134,MCAL-25822,MCAL-25730,MCAL-25729,MCAL-25728</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -2624,12 +2624,12 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Architecture,Design,Design,Design,Design,Design,Design,Architecture,Design,Design,Design,Design,Architecture,Architecture,Architecture,Architecture,Architecture,Design,Architecture</t>
+          <t>Architecture,Design,Design,Design,Design,Design,Design,Architecture,Design,Design,Design,Design,Architecture,Architecture,Architecture,Design,Architecture,Architecture,Architecture</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>MCAL-25189,MCAL-25530,MCAL-25533,MCAL-25534,MCAL-25535,MCAL-25538,MCAL-25540,MCAL-25190,MCAL-25531,MCAL-25532,MCAL-25537,MCAL-25539,MCAL-28233,MCAL-25192,MCAL-25194,MCAL-25195,MCAL-25191,MCAL-25536,MCAL-25193</t>
+          <t>MCAL-25189,MCAL-25530,MCAL-25533,MCAL-25534,MCAL-25535,MCAL-25538,MCAL-25540,MCAL-25190,MCAL-25531,MCAL-25532,MCAL-25537,MCAL-25539,MCAL-28233,MCAL-25192,MCAL-25194,MCAL-25536,MCAL-25195,MCAL-25191,MCAL-25193</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -2822,12 +2822,12 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Architecture,Design,Architecture,Design,Architecture,Architecture,Architecture,Design,Design,Architecture,Architecture,Design,Design,Design</t>
+          <t>Architecture,Design,Architecture,Design,Architecture,Design,Design,Architecture,Architecture,Design,Architecture,Architecture,Design,Design</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>MCAL-25190,MCAL-25592,MCAL-25191,MCAL-25590,MCAL-25192,MCAL-25194,MCAL-25195,MCAL-25591,MCAL-25688,MCAL-25193,MCAL-25189,MCAL-25690,MCAL-25691,MCAL-25689</t>
+          <t>MCAL-25190,MCAL-25592,MCAL-25191,MCAL-25590,MCAL-25195,MCAL-25591,MCAL-25688,MCAL-25193,MCAL-25189,MCAL-25690,MCAL-25192,MCAL-25194,MCAL-25691,MCAL-25689</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -5074,7 +5074,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>MCAL-24888,MCAL-25066,MCAL-25068,MCAL-25060,MCAL-25061,MCAL-25051,MCAL-25111,MCAL-28292,MCAL-24983,MCAL-24951,MCAL-25059,MCAL-25065,MCAL-24956</t>
+          <t>MCAL-24888,MCAL-25066,MCAL-25068,MCAL-25060,MCAL-25061,MCAL-25051,MCAL-25111,MCAL-28292,MCAL-24983,MCAL-24951,MCAL-24956,MCAL-25065,MCAL-25059</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">

</xml_diff>